<commit_message>
Requirements actualizados y listo para la nube
</commit_message>
<xml_diff>
--- a/obras.xlsx
+++ b/obras.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://termofrio365-my.sharepoint.com/personal/lzuniga_termofrio_cl/Documents/Control Taller 2025/SISTEMA_INTEGRAL_TERMOFRIO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="8_{6D6AE284-D4B4-4150-B274-F67A0E6CC822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{121DAFB7-0614-40EF-BB8B-A9508BDEBC71}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{6D6AE284-D4B4-4150-B274-F67A0E6CC822}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C56EA3FE-3CA8-4C3E-ADDC-BE39023044B3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{82446C5C-DF1E-4136-8F16-D06B8C8B0D1D}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="78">
   <si>
     <t>TF</t>
   </si>
@@ -261,6 +261,12 @@
   </si>
   <si>
     <t>EXTRAS 4-03-002</t>
+  </si>
+  <si>
+    <t>TF-13912 ECOEGAÑA- PLACA COMERCIAL- LOCALES DE COMIDA</t>
+  </si>
+  <si>
+    <t>2-14-022</t>
   </si>
 </sst>
 </file>
@@ -370,6 +376,7 @@
       <sheetName val="Calendario"/>
       <sheetName val="Seguimiento OC"/>
       <sheetName val="Hoja1"/>
+      <sheetName val="Control Procesos 2025"/>
     </sheetNames>
     <sheetDataSet>
       <sheetData sheetId="0"/>
@@ -397,6 +404,7 @@
       <sheetData sheetId="22"/>
       <sheetData sheetId="23"/>
       <sheetData sheetId="24"/>
+      <sheetData sheetId="25" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -700,7 +708,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04FFFAEB-562E-4C1D-87BB-DC6640D9CC9D}">
   <sheetPr codeName="Hoja4"/>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="1"/>
@@ -1412,6 +1420,17 @@
         <v>65</v>
       </c>
     </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>13912</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>